<commit_message>
lots of small changes
</commit_message>
<xml_diff>
--- a/ACQUISITION/Acquisition planning.xlsx
+++ b/ACQUISITION/Acquisition planning.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -510,213 +510,213 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Start here: ACQUISITION/ideal-business-fit.md — operator fit map before any listing search.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>TAB GUIDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>01_Archetype_Scorecard — vertical fit with formula-driven weighted scores</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>02_Target_Size_Bands — SDE/EBITDA/EV bands and affordability calculator</t>
+          <t>01_Archetype_Scorecard — vertical fit, Fit class (Buy/Conditional/Never), weighted Tier</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>03_Operator_Readiness — financing, runway, willingness gates</t>
+          <t>02_Target_Size_Bands — SDE/EBITDA/EV bands and affordability calculator</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>04_Deal_Pipeline — real listings only</t>
+          <t>03_Operator_Readiness — financing, runway, willingness gates</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>05_Deal_Scorecard — per-deal weighted score + Pursue/Watch/Kill</t>
+          <t>04_Deal_Pipeline — real listings only</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>06_Business_Risk_Diligence — personnel, ops, customer, revenue quality</t>
+          <t>05_Deal_Scorecard — per-deal weighted score + Day-to-day litmus gate + Pursue/Watch/Kill</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>07_Diligence_Memo — one-page memo template per deal</t>
+          <t>06_Business_Risk_Diligence — personnel, ops, customer, revenue quality</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>08_Time_Budget — weekly hours across Path A, Path B, acquisition</t>
+          <t>07_Diligence_Memo — one-page memo template per deal</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09_Decision_Log — dated pass/kill decisions</t>
+          <t>08_Time_Budget — weekly hours across Path A, Path B, acquisition</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>09_Decision_Log — dated pass/kill decisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>10_Ownership_Stress — financial stress + profile litmus before Pursue</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>THREE GATES (all required)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>1. Business you could improve</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2. Business you could realistically buy</t>
+          <t>1. Business you could improve</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>2. Business you could realistically buy</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>3. Business you would operate for 3 years</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>DEAL SCORECARD WEIGHTS</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Operator fit — 25%</t>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>ARCHETYPE VS TIER</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>AI/product leverage — 20%</t>
+          <t>Archetype = deal shape (SaaS with ops mess, services + workflow, etc.) — see acquisition_archetypes.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Financial feasibility — 25%</t>
+          <t>Tier = workbook vertical weighted score (Tier 1/2/3). High Tier does NOT override Fit class Never or day-to-day litmus NO.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Owner dependence / transition — 15%</t>
+          <t>Fit class = operator-fit judgment (Buy / Conditional / Never) — see ideal-business-fit.md</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Operating enjoyment — 10%</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Strategic conflict risk — 5%</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>DEAL SCORECARD WEIGHTS</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Operator fit — 25%</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>LABELS: Pursue (score &gt;= 3.5 and gates pass) | Watch (2.5-3.4 or missing data) | Kill (&lt; 2.5 or hard fail)</t>
+          <t>AI/product leverage — 20%</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Financial feasibility — 25%</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>FORMULA APPENDIX (Google Sheets-safe)</t>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Owner dependence / transition — 15%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Weighted total: =SUMPRODUCT(weights, scores) / SUM(weights)</t>
+          <t>Operating enjoyment — 10%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Decision label: =IF(AND(score&gt;=3.5, gates="YES"), "Pursue", IF(OR(score&lt;2.5, hardFail="YES"), "Kill", "Watch"))</t>
+          <t>Strategic conflict risk — 5%</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>DSCR: =IF(debtService=0, "", normalizedEBITDA/debtService)</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>EV/SDE: =IF(SDE=0, "", askingPrice/SDE)</t>
+          <t>LABELS: Pursue (score &gt;= 3.5 and gates pass) | Watch (2.5-3.4 or missing data) | Kill (&lt; 2.5 or hard fail)</t>
         </is>
       </c>
     </row>
@@ -726,35 +726,35 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>KILL RULES — pause search if:</t>
+          <t>FORMULA APPENDIX (Google Sheets-safe)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>• Acquisition &gt; 8 hrs/wk for 2 weeks while Path B outbound &lt; 5 hrs/wk</t>
+          <t>Weighted total: =SUMPRODUCT(weights, scores) / SUM(weights)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>• New domain listing outside ops-AI/logistics (month-5 relapse)</t>
+          <t>Decision label: =IF(AND(score&gt;=3.5, gates="YES"), "Pursue", IF(OR(score&lt;2.5, hardFail="YES"), "Kill", "Watch"))</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>• LOI without financing pre-approval</t>
+          <t>DSCR: =IF(debtService=0, "", normalizedEBITDA/debtService)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>• Deal fails all three gates</t>
+          <t>EV/SDE: =IF(SDE=0, "", askingPrice/SDE)</t>
         </is>
       </c>
     </row>
@@ -762,9 +762,61 @@
       <c r="A43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>See ACQUISITION/README.md and ownership-challenges.md for full rules.</t>
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>KILL RULES — pause search if:</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>1. Acquisition &gt; 8 hrs/wk for 2 weeks while Path B outbound &lt; 5 hrs/wk</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2. New domain listing outside ops-AI/logistics (month-5 relapse)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>3. LOI without financing pre-approval and 12-month runway model</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>4. Deal fails all three gates (improve / buy / operate 3yr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>5. Path B offer accepted — acquisition pauses 6 months minimum</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>6. Quotely hits 5+ paying operators — re-evaluate whether acquisition dilutes Path A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>See ACQUISITION/README.md, ideal-business-fit.md, and ownership-challenges.md for full rules.</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1468,8 +1520,9 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1525,10 +1578,15 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
+          <t>Fit class</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1599,7 +1657,12 @@
         <f>ROUND((B3*$B$2+C3*$C$2+D3*$D$2+E3*$E$2+F3*$F$2+G3*$G$2+(10-H3)*$H$2+(10-I3)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K3" s="5">
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Conditional</t>
+        </is>
+      </c>
+      <c r="L3" s="5">
         <f>IF(J3&gt;=7.5,"Tier 1",IF(J3&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1638,7 +1701,12 @@
         <f>ROUND((B4*$B$2+C4*$C$2+D4*$D$2+E4*$E$2+F4*$F$2+G4*$G$2+(10-H4)*$H$2+(10-I4)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="L4" s="5">
         <f>IF(J4&gt;=7.5,"Tier 1",IF(J4&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1677,7 +1745,12 @@
         <f>ROUND((B5*$B$2+C5*$C$2+D5*$D$2+E5*$E$2+F5*$F$2+G5*$G$2+(10-H5)*$H$2+(10-I5)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="L5" s="5">
         <f>IF(J5&gt;=7.5,"Tier 1",IF(J5&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1716,7 +1789,12 @@
         <f>ROUND((B6*$B$2+C6*$C$2+D6*$D$2+E6*$E$2+F6*$F$2+G6*$G$2+(10-H6)*$H$2+(10-I6)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Conditional</t>
+        </is>
+      </c>
+      <c r="L6" s="5">
         <f>IF(J6&gt;=7.5,"Tier 1",IF(J6&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1755,7 +1833,12 @@
         <f>ROUND((B7*$B$2+C7*$C$2+D7*$D$2+E7*$E$2+F7*$F$2+G7*$G$2+(10-H7)*$H$2+(10-I7)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="L7" s="5">
         <f>IF(J7&gt;=7.5,"Tier 1",IF(J7&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1794,7 +1877,12 @@
         <f>ROUND((B8*$B$2+C8*$C$2+D8*$D$2+E8*$E$2+F8*$F$2+G8*$G$2+(10-H8)*$H$2+(10-I8)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>Conditional</t>
+        </is>
+      </c>
+      <c r="L8" s="5">
         <f>IF(J8&gt;=7.5,"Tier 1",IF(J8&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1833,7 +1921,12 @@
         <f>ROUND((B9*$B$2+C9*$C$2+D9*$D$2+E9*$E$2+F9*$F$2+G9*$G$2+(10-H9)*$H$2+(10-I9)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="L9" s="5">
         <f>IF(J9&gt;=7.5,"Tier 1",IF(J9&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1872,7 +1965,12 @@
         <f>ROUND((B10*$B$2+C10*$C$2+D10*$D$2+E10*$E$2+F10*$F$2+G10*$G$2+(10-H10)*$H$2+(10-I10)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="L10" s="5">
         <f>IF(J10&gt;=7.5,"Tier 1",IF(J10&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1911,7 +2009,12 @@
         <f>ROUND((B11*$B$2+C11*$C$2+D11*$D$2+E11*$E$2+F11*$F$2+G11*$G$2+(10-H11)*$H$2+(10-I11)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="L11" s="5">
         <f>IF(J11&gt;=7.5,"Tier 1",IF(J11&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1950,7 +2053,12 @@
         <f>ROUND((B12*$B$2+C12*$C$2+D12*$D$2+E12*$E$2+F12*$F$2+G12*$G$2+(10-H12)*$H$2+(10-I12)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K12" s="5">
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="L12" s="5">
         <f>IF(J12&gt;=7.5,"Tier 1",IF(J12&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -1989,7 +2097,12 @@
         <f>ROUND((B13*$B$2+C13*$C$2+D13*$D$2+E13*$E$2+F13*$F$2+G13*$G$2+(10-H13)*$H$2+(10-I13)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K13" s="5">
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="L13" s="5">
         <f>IF(J13&gt;=7.5,"Tier 1",IF(J13&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -2028,7 +2141,12 @@
         <f>ROUND((B14*$B$2+C14*$C$2+D14*$D$2+E14*$E$2+F14*$F$2+G14*$G$2+(10-H14)*$H$2+(10-I14)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="L14" s="5">
         <f>IF(J14&gt;=7.5,"Tier 1",IF(J14&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -2067,7 +2185,12 @@
         <f>ROUND((B15*$B$2+C15*$C$2+D15*$D$2+E15*$E$2+F15*$F$2+G15*$G$2+(10-H15)*$H$2+(10-I15)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="L15" s="5">
         <f>IF(J15&gt;=7.5,"Tier 1",IF(J15&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -2106,7 +2229,12 @@
         <f>ROUND((B16*$B$2+C16*$C$2+D16*$D$2+E16*$E$2+F16*$F$2+G16*$G$2+(10-H16)*$H$2+(10-I16)*$I$2)/SUM($B$2:$I$2),1)</f>
         <v/>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="L16" s="5">
         <f>IF(J16&gt;=7.5,"Tier 1",IF(J16&gt;=5.5,"Tier 2","Tier 3"))</f>
         <v/>
       </c>
@@ -2436,6 +2564,50 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="14">
+    <dataValidation sqref="K3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buy,Conditional,Never,Review"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3752,16 +3924,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3827,30 +4000,35 @@
       </c>
       <c r="M1" s="4" t="inlineStr">
         <is>
+          <t>Day-to-day litmus?</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
           <t>Financing documented?</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>Path B displaced?</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>Risk red flags (#)</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>All gates pass?</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>Hard fail?</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
@@ -3904,20 +4082,21 @@
       <c r="L3" s="6" t="n"/>
       <c r="M3" s="6" t="n"/>
       <c r="N3" s="6" t="n"/>
-      <c r="O3" s="5">
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="5">
         <f>'06_Business_Risk_Diligence'!V3</f>
         <v/>
       </c>
-      <c r="P3" s="5">
-        <f>IF(COUNTIF(J3:N3,"NO")&gt;0,"NO","YES")</f>
-        <v/>
-      </c>
       <c r="Q3" s="5">
-        <f>IF(OR(N3="YES",O3&gt;=3,M3="NO"),"YES","NO")</f>
+        <f>IF(COUNTIF(J3:O3,"NO")&gt;0,"NO","YES")</f>
         <v/>
       </c>
       <c r="R3" s="5">
-        <f>IF(AND(I3&gt;=3.5,P3="YES",Q3="NO"),"Pursue",IF(OR(I3&lt;2.5,Q3="YES"),"Kill","Watch"))</f>
+        <f>IF(OR(M3="NO",N3="NO",O3="YES",P3&gt;=3),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="S3" s="5">
+        <f>IF(AND(I3&gt;=3.5,Q3="YES",R3="NO"),"Pursue",IF(OR(I3&lt;2.5,R3="YES"),"Kill","Watch"))</f>
         <v/>
       </c>
     </row>
@@ -3943,20 +4122,21 @@
       <c r="L4" s="6" t="n"/>
       <c r="M4" s="6" t="n"/>
       <c r="N4" s="6" t="n"/>
-      <c r="O4" s="5">
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="5">
         <f>'06_Business_Risk_Diligence'!V4</f>
         <v/>
       </c>
-      <c r="P4" s="5">
-        <f>IF(COUNTIF(J4:N4,"NO")&gt;0,"NO","YES")</f>
-        <v/>
-      </c>
       <c r="Q4" s="5">
-        <f>IF(OR(N4="YES",O4&gt;=3,M4="NO"),"YES","NO")</f>
+        <f>IF(COUNTIF(J4:O4,"NO")&gt;0,"NO","YES")</f>
         <v/>
       </c>
       <c r="R4" s="5">
-        <f>IF(AND(I4&gt;=3.5,P4="YES",Q4="NO"),"Pursue",IF(OR(I4&lt;2.5,Q4="YES"),"Kill","Watch"))</f>
+        <f>IF(OR(M4="NO",N4="NO",O4="YES",P4&gt;=3),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="S4" s="5">
+        <f>IF(AND(I4&gt;=3.5,Q4="YES",R4="NO"),"Pursue",IF(OR(I4&lt;2.5,R4="YES"),"Kill","Watch"))</f>
         <v/>
       </c>
     </row>
@@ -3982,20 +4162,21 @@
       <c r="L5" s="6" t="n"/>
       <c r="M5" s="6" t="n"/>
       <c r="N5" s="6" t="n"/>
-      <c r="O5" s="5">
+      <c r="O5" s="6" t="n"/>
+      <c r="P5" s="5">
         <f>'06_Business_Risk_Diligence'!V5</f>
         <v/>
       </c>
-      <c r="P5" s="5">
-        <f>IF(COUNTIF(J5:N5,"NO")&gt;0,"NO","YES")</f>
-        <v/>
-      </c>
       <c r="Q5" s="5">
-        <f>IF(OR(N5="YES",O5&gt;=3,M5="NO"),"YES","NO")</f>
+        <f>IF(COUNTIF(J5:O5,"NO")&gt;0,"NO","YES")</f>
         <v/>
       </c>
       <c r="R5" s="5">
-        <f>IF(AND(I5&gt;=3.5,P5="YES",Q5="NO"),"Pursue",IF(OR(I5&lt;2.5,Q5="YES"),"Kill","Watch"))</f>
+        <f>IF(OR(M5="NO",N5="NO",O5="YES",P5&gt;=3),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="S5" s="5">
+        <f>IF(AND(I5&gt;=3.5,Q5="YES",R5="NO"),"Pursue",IF(OR(I5&lt;2.5,R5="YES"),"Kill","Watch"))</f>
         <v/>
       </c>
     </row>
@@ -4021,20 +4202,21 @@
       <c r="L6" s="6" t="n"/>
       <c r="M6" s="6" t="n"/>
       <c r="N6" s="6" t="n"/>
-      <c r="O6" s="5">
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="5">
         <f>'06_Business_Risk_Diligence'!V6</f>
         <v/>
       </c>
-      <c r="P6" s="5">
-        <f>IF(COUNTIF(J6:N6,"NO")&gt;0,"NO","YES")</f>
-        <v/>
-      </c>
       <c r="Q6" s="5">
-        <f>IF(OR(N6="YES",O6&gt;=3,M6="NO"),"YES","NO")</f>
+        <f>IF(COUNTIF(J6:O6,"NO")&gt;0,"NO","YES")</f>
         <v/>
       </c>
       <c r="R6" s="5">
-        <f>IF(AND(I6&gt;=3.5,P6="YES",Q6="NO"),"Pursue",IF(OR(I6&lt;2.5,Q6="YES"),"Kill","Watch"))</f>
+        <f>IF(OR(M6="NO",N6="NO",O6="YES",P6&gt;=3),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="S6" s="5">
+        <f>IF(AND(I6&gt;=3.5,Q6="YES",R6="NO"),"Pursue",IF(OR(I6&lt;2.5,R6="YES"),"Kill","Watch"))</f>
         <v/>
       </c>
     </row>
@@ -4060,20 +4242,21 @@
       <c r="L7" s="6" t="n"/>
       <c r="M7" s="6" t="n"/>
       <c r="N7" s="6" t="n"/>
-      <c r="O7" s="5">
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="5">
         <f>'06_Business_Risk_Diligence'!V7</f>
         <v/>
       </c>
-      <c r="P7" s="5">
-        <f>IF(COUNTIF(J7:N7,"NO")&gt;0,"NO","YES")</f>
-        <v/>
-      </c>
       <c r="Q7" s="5">
-        <f>IF(OR(N7="YES",O7&gt;=3,M7="NO"),"YES","NO")</f>
+        <f>IF(COUNTIF(J7:O7,"NO")&gt;0,"NO","YES")</f>
         <v/>
       </c>
       <c r="R7" s="5">
-        <f>IF(AND(I7&gt;=3.5,P7="YES",Q7="NO"),"Pursue",IF(OR(I7&lt;2.5,Q7="YES"),"Kill","Watch"))</f>
+        <f>IF(OR(M7="NO",N7="NO",O7="YES",P7&gt;=3),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="S7" s="5">
+        <f>IF(AND(I7&gt;=3.5,Q7="YES",R7="NO"),"Pursue",IF(OR(I7&lt;2.5,R7="YES"),"Kill","Watch"))</f>
         <v/>
       </c>
     </row>
@@ -4083,35 +4266,35 @@
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="J3:N3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J3:O3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"YES,NO,Unknown"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:H4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="J4:N4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:O4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"YES,NO,Unknown"</formula1>
     </dataValidation>
     <dataValidation sqref="C5:H5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="J5:N5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J5:O5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"YES,NO,Unknown"</formula1>
     </dataValidation>
     <dataValidation sqref="C6:H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="J6:N6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J6:O6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"YES,NO,Unknown"</formula1>
     </dataValidation>
     <dataValidation sqref="C7:H7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="J7:N7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J7:O7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"YES,NO,Unknown"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>